<commit_message>
reworked input excel data
</commit_message>
<xml_diff>
--- a/Input/Einkauf Kiosk  01.11.23.xlsx
+++ b/Input/Einkauf Kiosk  01.11.23.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\R Packages\Kinoklub\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A12B0C0A-E41D-4BC1-AC6C-D74713FCFA60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62A4CB17-1311-4BE3-8DF6-76FE6F6936EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B11F654B-1788-4E85-B872-7BAC8A50C723}"/>
+    <workbookView xWindow="12885" yWindow="4695" windowWidth="12240" windowHeight="15150" xr2:uid="{B11F654B-1788-4E85-B872-7BAC8A50C723}"/>
   </bookViews>
   <sheets>
     <sheet name="Angebot" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="81">
   <si>
     <t>Schüwo</t>
   </si>
@@ -128,9 +128,6 @@
     <t>Popcorn Sweet&amp;Salty</t>
   </si>
   <si>
-    <t>Einkaufspreis gesamt</t>
-  </si>
-  <si>
     <t>Quöllfrisch</t>
   </si>
   <si>
@@ -230,9 +227,6 @@
     <t>Einkaufs- preis</t>
   </si>
   <si>
-    <t>Anzahl Bestellung Feb 2024</t>
-  </si>
-  <si>
     <t>Glacé Caramel</t>
   </si>
   <si>
@@ -279,6 +273,12 @@
   </si>
   <si>
     <t>Weisser Kaffee</t>
+  </si>
+  <si>
+    <t>10cl</t>
+  </si>
+  <si>
+    <t>30cl</t>
   </si>
 </sst>
 </file>
@@ -400,10 +400,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -431,7 +430,7 @@
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="20">
+  <dxfs count="16">
     <dxf>
       <font>
         <b/>
@@ -466,8 +465,12 @@
         <bottom style="hair">
           <color indexed="64"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
+        <vertical style="hair">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="hair">
+          <color indexed="64"/>
+        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -567,6 +570,7 @@
       </font>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;CHF&quot;\ #,##0.00"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="hair">
           <color indexed="64"/>
@@ -645,85 +649,6 @@
       </font>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;CHF&quot;\ #,##0.00"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="&quot;CHF&quot;\ #,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;CHF&quot;\ #,##0.00"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="hair">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="hair">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
       <border diagonalUp="0" diagonalDown="0">
         <left style="hair">
           <color indexed="64"/>
@@ -803,21 +728,17 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{920C96DA-BD94-48CE-B13B-7B1D665A1F1C}" name="Table1" displayName="Table1" ref="A1:I38" headerRowDxfId="19" totalsRowDxfId="18">
-  <autoFilter ref="A1:I38" xr:uid="{920C96DA-BD94-48CE-B13B-7B1D665A1F1C}"/>
-  <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{E8635A23-EB85-4436-9D20-6BDBA55F1730}" name="Artikel" totalsRowLabel="Total" dataDxfId="17" totalsRowDxfId="16"/>
-    <tableColumn id="4" xr3:uid="{3577DE02-0CD1-4A73-82D1-7EE95A59F5D7}" name="Artikelname Kassensystem" dataDxfId="15" totalsRowDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{76440182-93E9-4612-87D8-CE2EBC73BDDF}" name="Verkaufs-preis" totalsRowFunction="sum" dataDxfId="13" totalsRowDxfId="12"/>
-    <tableColumn id="8" xr3:uid="{B2930651-661A-4264-8410-185C3D54A8C7}" name="Menge" dataDxfId="11" totalsRowDxfId="10"/>
-    <tableColumn id="6" xr3:uid="{AC0A2B1B-F4FB-4E77-BAD2-DD5CBF1419AB}" name="Einkaufs- preis" totalsRowFunction="sum" dataDxfId="9" totalsRowDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{35E0FA36-7D3F-4BDD-9461-90D996CC4D33}" name="Lieferant" dataDxfId="7" totalsRowDxfId="6"/>
-    <tableColumn id="7" xr3:uid="{506E2FE9-BDDF-4C71-B77C-D5359CF307ED}" name="Gewinn" totalsRowFunction="sum" dataDxfId="5" totalsRowDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{920C96DA-BD94-48CE-B13B-7B1D665A1F1C}" name="Table1" displayName="Table1" ref="A1:G38" headerRowDxfId="15" totalsRowDxfId="14">
+  <autoFilter ref="A1:G38" xr:uid="{920C96DA-BD94-48CE-B13B-7B1D665A1F1C}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{E8635A23-EB85-4436-9D20-6BDBA55F1730}" name="Artikel" totalsRowLabel="Total" dataDxfId="13" totalsRowDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{3577DE02-0CD1-4A73-82D1-7EE95A59F5D7}" name="Artikelname Kassensystem" dataDxfId="11" totalsRowDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{76440182-93E9-4612-87D8-CE2EBC73BDDF}" name="Verkaufs-preis" totalsRowFunction="sum" dataDxfId="9" totalsRowDxfId="8"/>
+    <tableColumn id="8" xr3:uid="{B2930651-661A-4264-8410-185C3D54A8C7}" name="Menge" dataDxfId="7" totalsRowDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{AC0A2B1B-F4FB-4E77-BAD2-DD5CBF1419AB}" name="Einkaufs- preis" totalsRowFunction="sum" dataDxfId="5" totalsRowDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{35E0FA36-7D3F-4BDD-9461-90D996CC4D33}" name="Lieferant" dataDxfId="3" totalsRowDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{506E2FE9-BDDF-4C71-B77C-D5359CF307ED}" name="Gewinn" totalsRowFunction="sum" dataDxfId="1" totalsRowDxfId="0">
       <calculatedColumnFormula>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="10" xr3:uid="{1164AC8E-A4BE-4CBA-B422-27C4A81D46E1}" name="Anzahl Bestellung Feb 2024" dataDxfId="3" totalsRowDxfId="2"/>
-    <tableColumn id="11" xr3:uid="{2DB050A1-5923-496C-9705-265C74DA448E}" name="Einkaufspreis gesamt" totalsRowFunction="sum" dataDxfId="1" totalsRowDxfId="0">
-      <calculatedColumnFormula>Table1[[#This Row],[Anzahl Bestellung Feb 2024]]*Table1[[#This Row],[Einkaufs- preis]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1121,1109 +1042,922 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A677428D-B810-4F63-BFBD-79DB0D9DB708}">
-  <dimension ref="A1:I38"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="33.85546875" customWidth="1"/>
-    <col min="3" max="3" width="11.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.28515625" style="7" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.28515625" style="7" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.28515625" style="8" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.42578125" customWidth="1"/>
-    <col min="9" max="9" width="13" style="8" customWidth="1"/>
+    <col min="7" max="7" width="10.28515625" style="7" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="15" customFormat="1" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+    <row r="1" spans="1:7" s="14" customFormat="1" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="12" t="s">
-        <v>49</v>
-      </c>
-      <c r="C1" s="13" t="s">
+      <c r="B1" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="E1" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="D1" s="14" t="s">
-        <v>37</v>
-      </c>
-      <c r="E1" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="G1" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="12" t="s">
-        <v>64</v>
-      </c>
-      <c r="I1" s="13" t="s">
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>30</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C2" s="5">
+      <c r="C2" s="4">
         <v>5</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="E2" s="5">
+      <c r="D2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="E2" s="4">
         <v>1.38</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="G2" s="5">
+      <c r="G2" s="4">
         <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
         <v>3.62</v>
       </c>
-      <c r="H2" s="1"/>
-      <c r="I2" s="5">
-        <f>Table1[[#This Row],[Anzahl Bestellung Feb 2024]]*Table1[[#This Row],[Einkaufs- preis]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C3" s="5">
+        <v>49</v>
+      </c>
+      <c r="C3" s="4">
         <v>5</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="E3" s="5">
+      <c r="D3" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="E3" s="4">
         <v>1.65</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="G3" s="5">
+      <c r="G3" s="4">
         <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
         <v>3.35</v>
       </c>
-      <c r="H3" s="1"/>
-      <c r="I3" s="5">
-        <f>Table1[[#This Row],[Anzahl Bestellung Feb 2024]]*Table1[[#This Row],[Einkaufs- preis]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="4">
         <v>7</v>
       </c>
-      <c r="D4" s="1"/>
-      <c r="E4" s="5">
+      <c r="D4" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="E4" s="4">
         <v>1.5</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="4">
         <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
         <v>5.5</v>
       </c>
-      <c r="H4" s="1"/>
-      <c r="I4" s="5">
-        <f>Table1[[#This Row],[Anzahl Bestellung Feb 2024]]*Table1[[#This Row],[Einkaufs- preis]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C5" s="4">
         <v>7</v>
       </c>
-      <c r="D5" s="1"/>
-      <c r="E5" s="5">
+      <c r="D5" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="E5" s="4">
         <v>1.4</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="G5" s="5">
+      <c r="G5" s="4">
         <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
         <v>5.6</v>
       </c>
-      <c r="H5" s="1"/>
-      <c r="I5" s="5">
-        <f>Table1[[#This Row],[Anzahl Bestellung Feb 2024]]*Table1[[#This Row],[Einkaufs- preis]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C6" s="4">
+        <v>4</v>
+      </c>
+      <c r="D6" s="1"/>
+      <c r="E6" s="4">
+        <v>0.15</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="G6" s="4">
+        <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
+        <v>3.85</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C6" s="5">
+      <c r="B7" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C7" s="4">
         <v>4</v>
       </c>
-      <c r="D6" s="1"/>
-      <c r="E6" s="5">
-        <v>0.15</v>
-      </c>
-      <c r="F6" s="1" t="s">
+      <c r="D7" s="1"/>
+      <c r="E7" s="10">
+        <v>0.5</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G6" s="5">
-        <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
-        <v>3.85</v>
-      </c>
-      <c r="H6" s="1"/>
-      <c r="I6" s="5">
-        <f>Table1[[#This Row],[Anzahl Bestellung Feb 2024]]*Table1[[#This Row],[Einkaufs- preis]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C7" s="5">
-        <v>4</v>
-      </c>
-      <c r="D7" s="1"/>
-      <c r="E7" s="11">
-        <v>0.5</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="G7" s="5">
+      <c r="G7" s="4">
         <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
         <v>3.5</v>
       </c>
-      <c r="H7" s="2"/>
-      <c r="I7" s="11">
-        <f>Table1[[#This Row],[Anzahl Bestellung Feb 2024]]*Table1[[#This Row],[Einkaufs- preis]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="5">
+      <c r="C8" s="4">
         <v>4.5</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="E8" s="5">
+        <v>38</v>
+      </c>
+      <c r="E8" s="4">
         <v>1.55</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="G8" s="5">
+      <c r="G8" s="4">
         <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
         <v>2.95</v>
       </c>
-      <c r="H8" s="1"/>
-      <c r="I8" s="5">
-        <f>Table1[[#This Row],[Anzahl Bestellung Feb 2024]]*Table1[[#This Row],[Einkaufs- preis]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="5">
+      <c r="C9" s="4">
         <v>4.5</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="E9" s="5">
+        <v>38</v>
+      </c>
+      <c r="E9" s="4">
         <v>1.55</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="G9" s="5">
+      <c r="G9" s="4">
         <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
         <v>2.95</v>
       </c>
-      <c r="H9" s="1"/>
-      <c r="I9" s="5">
-        <f>Table1[[#This Row],[Anzahl Bestellung Feb 2024]]*Table1[[#This Row],[Einkaufs- preis]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="5">
+      <c r="C10" s="4">
         <v>4</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="E10" s="5">
+        <v>39</v>
+      </c>
+      <c r="E10" s="4">
         <v>0.97</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="G10" s="5">
+      <c r="G10" s="4">
         <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
         <v>3.0300000000000002</v>
       </c>
-      <c r="H10" s="1"/>
-      <c r="I10" s="5">
-        <f>Table1[[#This Row],[Anzahl Bestellung Feb 2024]]*Table1[[#This Row],[Einkaufs- preis]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="5">
+      <c r="C11" s="4">
         <v>4</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="E11" s="5">
+        <v>39</v>
+      </c>
+      <c r="E11" s="4">
         <v>0.97</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="G11" s="5">
+      <c r="G11" s="4">
         <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
         <v>3.0300000000000002</v>
       </c>
-      <c r="H11" s="1"/>
-      <c r="I11" s="5">
-        <f>Table1[[#This Row],[Anzahl Bestellung Feb 2024]]*Table1[[#This Row],[Einkaufs- preis]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="5">
+      <c r="C12" s="4">
         <v>2</v>
       </c>
-      <c r="D12" s="1"/>
-      <c r="E12" s="11">
+      <c r="D12" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="E12" s="10">
         <v>0.3</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="G12" s="5">
+        <v>33</v>
+      </c>
+      <c r="G12" s="4">
         <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
         <v>1.7</v>
       </c>
-      <c r="H12" s="2"/>
-      <c r="I12" s="11">
-        <f>Table1[[#This Row],[Anzahl Bestellung Feb 2024]]*Table1[[#This Row],[Einkaufs- preis]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>9</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="C13" s="5">
+        <v>52</v>
+      </c>
+      <c r="C13" s="4">
         <v>5</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E13" s="5">
+        <v>37</v>
+      </c>
+      <c r="E13" s="4">
         <v>1.1499999999999999</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="G13" s="5">
+      <c r="G13" s="4">
         <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
         <v>3.85</v>
       </c>
-      <c r="H13" s="1"/>
-      <c r="I13" s="5">
-        <f>Table1[[#This Row],[Anzahl Bestellung Feb 2024]]*Table1[[#This Row],[Einkaufs- preis]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="C14" s="5">
+        <v>53</v>
+      </c>
+      <c r="C14" s="4">
         <v>5</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E14" s="5">
+        <v>37</v>
+      </c>
+      <c r="E14" s="4">
         <v>1.1499999999999999</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="G14" s="5">
+      <c r="G14" s="4">
         <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
         <v>3.85</v>
       </c>
-      <c r="H14" s="1"/>
-      <c r="I14" s="5">
-        <f>Table1[[#This Row],[Anzahl Bestellung Feb 2024]]*Table1[[#This Row],[Einkaufs- preis]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>23</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C15" s="5">
+      <c r="C15" s="4">
         <v>6</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E15" s="5">
+        <v>40</v>
+      </c>
+      <c r="E15" s="4">
         <v>1.44</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="G15" s="5">
+      <c r="G15" s="4">
         <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
         <v>4.5600000000000005</v>
       </c>
-      <c r="H15" s="1"/>
-      <c r="I15" s="5">
-        <f>Table1[[#This Row],[Anzahl Bestellung Feb 2024]]*Table1[[#This Row],[Einkaufs- preis]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C16" s="5">
+      <c r="C16" s="4">
         <v>5</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E16" s="5">
+        <v>37</v>
+      </c>
+      <c r="E16" s="4">
         <v>1.1200000000000001</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="G16" s="5">
+      <c r="G16" s="4">
         <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
         <v>3.88</v>
       </c>
-      <c r="H16" s="1"/>
-      <c r="I16" s="5">
-        <f>Table1[[#This Row],[Anzahl Bestellung Feb 2024]]*Table1[[#This Row],[Einkaufs- preis]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C17" s="5">
+      <c r="C17" s="4">
         <v>6</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E17" s="5">
+        <v>40</v>
+      </c>
+      <c r="E17" s="4">
         <v>1.44</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="G17" s="5">
+      <c r="G17" s="4">
         <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
         <v>4.5600000000000005</v>
       </c>
-      <c r="H17" s="1"/>
-      <c r="I17" s="5">
-        <f>Table1[[#This Row],[Anzahl Bestellung Feb 2024]]*Table1[[#This Row],[Einkaufs- preis]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>25</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C18" s="5">
+      <c r="C18" s="4">
         <v>6</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E18" s="5">
+        <v>40</v>
+      </c>
+      <c r="E18" s="4">
         <v>1.44</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="G18" s="5">
+      <c r="G18" s="4">
         <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
         <v>4.5600000000000005</v>
       </c>
-      <c r="H18" s="1"/>
-      <c r="I18" s="5">
-        <f>Table1[[#This Row],[Anzahl Bestellung Feb 2024]]*Table1[[#This Row],[Einkaufs- preis]]</f>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C19" s="5">
+        <v>5</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E19" s="5">
+        <v>1.03</v>
+      </c>
+      <c r="F19" s="3" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="C19" s="6">
+      <c r="G19" s="5">
+        <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
+        <v>3.9699999999999998</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C20" s="6">
         <v>5</v>
       </c>
-      <c r="D19" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E19" s="6">
-        <v>1.03</v>
-      </c>
-      <c r="F19" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="G19" s="6">
-        <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
-        <v>3.9699999999999998</v>
-      </c>
-      <c r="H19" s="4"/>
-      <c r="I19" s="6">
-        <f>Table1[[#This Row],[Anzahl Bestellung Feb 2024]]*Table1[[#This Row],[Einkaufs- preis]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C20" s="7">
-        <v>5</v>
-      </c>
       <c r="D20" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="E20" s="7">
+        <v>45</v>
+      </c>
+      <c r="E20" s="6">
         <v>1.95</v>
       </c>
-      <c r="F20" s="3" t="s">
+      <c r="F20" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G20" s="5">
+      <c r="G20" s="4">
         <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
         <v>3.05</v>
       </c>
-      <c r="H20" s="3"/>
-      <c r="I20" s="7">
-        <f>Table1[[#This Row],[Anzahl Bestellung Feb 2024]]*Table1[[#This Row],[Einkaufs- preis]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>29</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C21" s="5">
+        <v>55</v>
+      </c>
+      <c r="C21" s="4">
         <v>5</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E21" s="5">
+        <v>46</v>
+      </c>
+      <c r="E21" s="4">
         <v>2.2000000000000002</v>
       </c>
       <c r="F21" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G21" s="5">
+      <c r="G21" s="4">
         <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
         <v>2.8</v>
       </c>
-      <c r="H21" s="1"/>
-      <c r="I21" s="5">
-        <f>Table1[[#This Row],[Anzahl Bestellung Feb 2024]]*Table1[[#This Row],[Einkaufs- preis]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="C22" s="5">
+        <v>54</v>
+      </c>
+      <c r="C22" s="4">
         <v>5</v>
       </c>
-      <c r="D22" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E22" s="5">
+      <c r="D22" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="E22" s="4">
         <v>0.4</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="G22" s="5">
+        <v>34</v>
+      </c>
+      <c r="G22" s="4">
         <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
         <v>4.5999999999999996</v>
       </c>
-      <c r="H22" s="1"/>
-      <c r="I22" s="5">
-        <f>Table1[[#This Row],[Anzahl Bestellung Feb 2024]]*Table1[[#This Row],[Einkaufs- preis]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C23" s="7">
+      <c r="C23" s="6">
         <v>5</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="E23" s="7">
+        <v>41</v>
+      </c>
+      <c r="E23" s="6">
         <v>4.17</v>
       </c>
-      <c r="F23" s="3" t="s">
+      <c r="F23" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G23" s="5">
+      <c r="G23" s="4">
         <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
         <v>0.83000000000000007</v>
       </c>
-      <c r="H23" s="3"/>
-      <c r="I23" s="7">
-        <f>Table1[[#This Row],[Anzahl Bestellung Feb 2024]]*Table1[[#This Row],[Einkaufs- preis]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C24" s="5">
+      <c r="C24" s="4">
         <v>3</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E24" s="5">
+        <v>42</v>
+      </c>
+      <c r="E24" s="4">
         <v>1.06</v>
       </c>
       <c r="F24" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G24" s="5">
+      <c r="G24" s="4">
         <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
         <v>1.94</v>
       </c>
-      <c r="H24" s="1"/>
-      <c r="I24" s="5">
-        <f>Table1[[#This Row],[Anzahl Bestellung Feb 2024]]*Table1[[#This Row],[Einkaufs- preis]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C25" s="5">
+      <c r="C25" s="4">
         <v>3</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="E25" s="5">
+        <v>43</v>
+      </c>
+      <c r="E25" s="4">
         <v>1.06</v>
       </c>
       <c r="F25" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G25" s="5">
+      <c r="G25" s="4">
         <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
         <v>1.94</v>
       </c>
-      <c r="H25" s="1"/>
-      <c r="I25" s="5">
-        <f>Table1[[#This Row],[Anzahl Bestellung Feb 2024]]*Table1[[#This Row],[Einkaufs- preis]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C26" s="5">
+      <c r="C26" s="4">
         <v>3</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="E26" s="5">
+      <c r="E26" s="4">
         <v>1.06</v>
       </c>
       <c r="F26" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G26" s="5">
+      <c r="G26" s="4">
         <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
         <v>1.94</v>
       </c>
-      <c r="H26" s="1"/>
-      <c r="I26" s="5">
-        <f>Table1[[#This Row],[Anzahl Bestellung Feb 2024]]*Table1[[#This Row],[Einkaufs- preis]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>18</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C27" s="5">
+      <c r="C27" s="4">
         <v>3</v>
       </c>
       <c r="D27" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="E27" s="5">
+      <c r="E27" s="4">
         <v>1.06</v>
       </c>
       <c r="F27" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G27" s="5">
+      <c r="G27" s="4">
         <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
         <v>1.94</v>
       </c>
-      <c r="H27" s="1"/>
-      <c r="I27" s="5">
-        <f>Table1[[#This Row],[Anzahl Bestellung Feb 2024]]*Table1[[#This Row],[Einkaufs- preis]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="B28" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="C28" s="6">
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="B28" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C28" s="5">
         <v>3</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E28" s="6">
+        <v>44</v>
+      </c>
+      <c r="E28" s="5">
         <v>0.99</v>
       </c>
-      <c r="F28" s="4" t="s">
+      <c r="F28" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G28" s="6">
+      <c r="G28" s="5">
         <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
         <v>2.0099999999999998</v>
       </c>
-      <c r="H28" s="4"/>
-      <c r="I28" s="6">
-        <f>Table1[[#This Row],[Anzahl Bestellung Feb 2024]]*Table1[[#This Row],[Einkaufs- preis]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="C29" s="5">
+        <v>56</v>
+      </c>
+      <c r="C29" s="4">
         <v>4</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="E29" s="5">
+        <v>47</v>
+      </c>
+      <c r="E29" s="4">
         <v>2.2999999999999998</v>
       </c>
       <c r="F29" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="G29" s="5">
+      <c r="G29" s="4">
         <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
         <v>1.7000000000000002</v>
       </c>
-      <c r="H29" s="1"/>
-      <c r="I29" s="5">
-        <f>Table1[[#This Row],[Anzahl Bestellung Feb 2024]]*Table1[[#This Row],[Einkaufs- preis]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="C30" s="5">
+        <v>57</v>
+      </c>
+      <c r="C30" s="4">
         <v>4</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="E30" s="5">
+        <v>47</v>
+      </c>
+      <c r="E30" s="4">
         <v>2.2999999999999998</v>
       </c>
       <c r="F30" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="G30" s="5">
+      <c r="G30" s="4">
         <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
         <v>1.7000000000000002</v>
       </c>
-      <c r="H30" s="1"/>
-      <c r="I30" s="5">
-        <f>Table1[[#This Row],[Anzahl Bestellung Feb 2024]]*Table1[[#This Row],[Einkaufs- preis]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C31" s="5">
+        <v>58</v>
+      </c>
+      <c r="C31" s="4">
         <v>4</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="E31" s="5">
+        <v>47</v>
+      </c>
+      <c r="E31" s="4">
         <v>2.2999999999999998</v>
       </c>
       <c r="F31" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="G31" s="5">
+      <c r="G31" s="4">
         <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
         <v>1.7000000000000002</v>
       </c>
-      <c r="H31" s="1"/>
-      <c r="I31" s="5">
-        <f>Table1[[#This Row],[Anzahl Bestellung Feb 2024]]*Table1[[#This Row],[Einkaufs- preis]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="C32" s="5">
+        <v>59</v>
+      </c>
+      <c r="C32" s="4">
         <v>4</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="E32" s="5">
+        <v>47</v>
+      </c>
+      <c r="E32" s="4">
         <v>2.2999999999999998</v>
       </c>
       <c r="F32" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="G32" s="5">
+      <c r="G32" s="4">
         <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
         <v>1.7000000000000002</v>
       </c>
-      <c r="H32" s="1"/>
-      <c r="I32" s="5">
-        <f>Table1[[#This Row],[Anzahl Bestellung Feb 2024]]*Table1[[#This Row],[Einkaufs- preis]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="C33" s="5">
+        <v>60</v>
+      </c>
+      <c r="C33" s="4">
         <v>4</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="E33" s="5">
+        <v>47</v>
+      </c>
+      <c r="E33" s="4">
         <v>2.2999999999999998</v>
       </c>
       <c r="F33" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="G33" s="5">
+      <c r="G33" s="4">
         <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
         <v>1.7000000000000002</v>
       </c>
-      <c r="H33" s="1"/>
-      <c r="I33" s="5">
-        <f>Table1[[#This Row],[Anzahl Bestellung Feb 2024]]*Table1[[#This Row],[Einkaufs- preis]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="16" t="s">
+    </row>
+    <row r="34" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="B34" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="C34" s="4">
+        <v>4</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E34" s="16">
+        <v>3</v>
+      </c>
+      <c r="F34" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="G34" s="16">
+        <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="B34" s="16" t="s">
+      <c r="B35" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="C35" s="4">
+        <v>4</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E35" s="16">
+        <v>3</v>
+      </c>
+      <c r="F35" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="G35" s="16">
+        <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" s="15" t="s">
         <v>71</v>
       </c>
-      <c r="C34" s="5">
+      <c r="B36" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="C36" s="4">
         <v>4</v>
       </c>
-      <c r="D34" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="E34" s="17">
+      <c r="D36" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E36" s="16">
         <v>3</v>
       </c>
-      <c r="F34" s="16" t="s">
-        <v>79</v>
-      </c>
-      <c r="G34" s="17">
+      <c r="F36" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="G36" s="16">
         <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
         <v>1</v>
       </c>
-      <c r="H34" s="16"/>
-      <c r="I34" s="17">
-        <f>Table1[[#This Row],[Anzahl Bestellung Feb 2024]]*Table1[[#This Row],[Einkaufs- preis]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A35" s="16" t="s">
-        <v>72</v>
-      </c>
-      <c r="B35" s="16" t="s">
-        <v>80</v>
-      </c>
-      <c r="C35" s="5">
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="B37" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="C37" s="4">
         <v>4</v>
       </c>
-      <c r="D35" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="E35" s="17">
+      <c r="D37" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E37" s="16">
         <v>3</v>
       </c>
-      <c r="F35" s="16" t="s">
-        <v>79</v>
-      </c>
-      <c r="G35" s="17">
+      <c r="F37" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="G37" s="16">
         <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
         <v>1</v>
       </c>
-      <c r="H35" s="16"/>
-      <c r="I35" s="17">
-        <f>Table1[[#This Row],[Anzahl Bestellung Feb 2024]]*Table1[[#This Row],[Einkaufs- preis]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A36" s="16" t="s">
-        <v>73</v>
-      </c>
-      <c r="B36" s="16" t="s">
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="C36" s="5">
+      <c r="B38" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="C38" s="4">
         <v>4</v>
       </c>
-      <c r="D36" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="E36" s="17">
+      <c r="D38" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E38" s="16">
         <v>3</v>
       </c>
-      <c r="F36" s="16" t="s">
-        <v>79</v>
-      </c>
-      <c r="G36" s="17">
+      <c r="F38" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="G38" s="16">
         <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
         <v>1</v>
-      </c>
-      <c r="H36" s="16"/>
-      <c r="I36" s="17">
-        <f>Table1[[#This Row],[Anzahl Bestellung Feb 2024]]*Table1[[#This Row],[Einkaufs- preis]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A37" s="16" t="s">
-        <v>75</v>
-      </c>
-      <c r="B37" s="16" t="s">
-        <v>77</v>
-      </c>
-      <c r="C37" s="5">
-        <v>4</v>
-      </c>
-      <c r="D37" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="E37" s="17">
-        <v>3</v>
-      </c>
-      <c r="F37" s="16" t="s">
-        <v>79</v>
-      </c>
-      <c r="G37" s="17">
-        <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
-        <v>1</v>
-      </c>
-      <c r="H37" s="16"/>
-      <c r="I37" s="17">
-        <f>Table1[[#This Row],[Anzahl Bestellung Feb 2024]]*Table1[[#This Row],[Einkaufs- preis]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A38" s="16" t="s">
-        <v>76</v>
-      </c>
-      <c r="B38" s="16" t="s">
-        <v>78</v>
-      </c>
-      <c r="C38" s="5">
-        <v>4</v>
-      </c>
-      <c r="D38" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="E38" s="17">
-        <v>3</v>
-      </c>
-      <c r="F38" s="16" t="s">
-        <v>79</v>
-      </c>
-      <c r="G38" s="17">
-        <f>Table1[[#This Row],[Verkaufs-preis]]-Table1[[#This Row],[Einkaufs- preis]]</f>
-        <v>1</v>
-      </c>
-      <c r="H38" s="16"/>
-      <c r="I38" s="17">
-        <f>Table1[[#This Row],[Anzahl Bestellung Feb 2024]]*Table1[[#This Row],[Einkaufs- preis]]</f>
-        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>